<commit_message>
LLM PR comments/fixes part 1
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="147">
   <si>
     <t>Translator notes</t>
   </si>
@@ -115,7 +115,7 @@
     <t>prns.prn.reprocessingSite</t>
   </si>
   <si>
-    <t>Reproccessing site</t>
+    <t>Reprocessing site</t>
   </si>
   <si>
     <t>Safle ailbrosesu</t>
@@ -374,6 +374,30 @@
   </si>
   <si>
     <t>Mae'r PRN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
+  </si>
+  <si>
+    <t>prns.prn.agency.ea</t>
+  </si>
+  <si>
+    <t>Environment Agency</t>
+  </si>
+  <si>
+    <t>prns.prn.agency.sepa</t>
+  </si>
+  <si>
+    <t>Scottish Environment Protection Agency</t>
+  </si>
+  <si>
+    <t>prns.prn.agency.niea</t>
+  </si>
+  <si>
+    <t>Northern Ireland Environment Agency</t>
+  </si>
+  <si>
+    <t>prns.prn.agency.nrw</t>
+  </si>
+  <si>
+    <t>Natural Resources Wales</t>
   </si>
   <si>
     <t>prns.prn.statusTypes.awaitingAcceptance</t>
@@ -826,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1757,7 +1781,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>129</v>
       </c>
@@ -1837,7 +1861,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>137</v>
       </c>
@@ -1857,8 +1881,88 @@
         <v>13</v>
       </c>
     </row>
+    <row r="55" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F54"/>
+  <autoFilter ref="A5:F58"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>